<commit_message>
reorganizando o workflow para como esta atualmente
</commit_message>
<xml_diff>
--- a/Execelteste/BaseRestricao.xlsx
+++ b/Execelteste/BaseRestricao.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobresser/Documents/Pessoal/PS/ws1/Execelteste/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joaobresser/Documents/Pessoal/PS/candidate_allocation/Execelteste/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE440334-4A60-6947-BB98-66C73FB0EAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C3CD529-F6BF-614B-9C96-3AA9914BDC4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Base" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="320">
   <si>
     <t>TimeStamp</t>
   </si>
@@ -983,9 +983,6 @@
   </si>
   <si>
     <t>A13 A9</t>
-  </si>
-  <si>
-    <t>Avaliador</t>
   </si>
   <si>
     <t>Sigla</t>
@@ -10228,14 +10225,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>316</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="C1" s="25" t="s">
         <v>317</v>
-      </c>
-      <c r="C1" s="25" t="s">
-        <v>318</v>
       </c>
       <c r="D1" s="7"/>
     </row>
@@ -10475,7 +10472,7 @@
         <v>297</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -10639,7 +10636,7 @@
         <v>53</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C16" s="21" t="s">
         <v>305</v>

</xml_diff>